<commit_message>
continued cleaning; structuring all data and getting readt for finalization of data before visualizations
</commit_message>
<xml_diff>
--- a/data/education/working/fod_earn_age.xlsx
+++ b/data/education/working/fod_earn_age.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,1460 +488,1404 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Field of Degree</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Population </t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Age 25 to 34</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Age 35 to 44</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Age 45 to 54 </t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Age 55 to 64 </t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
+          <t xml:space="preserve">Population 25 to 64 with a Bachelor's Degree or Higher with earnings </t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>74150</v>
+      </c>
+      <c r="C2" t="n">
+        <v>165.7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>60470</v>
+      </c>
+      <c r="E2" t="n">
+        <v>171.8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>79600</v>
+      </c>
+      <c r="G2" t="n">
+        <v>431.6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>86340</v>
+      </c>
+      <c r="I2" t="n">
+        <v>329.9</v>
+      </c>
+      <c r="J2" t="n">
+        <v>81580</v>
+      </c>
+      <c r="K2" t="n">
+        <v>350.3</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimate </t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOE </t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimate </t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOE </t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimate </t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOE </t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimate </t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOE </t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimate </t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOE </t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Science and Engineering Degrees </t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Population 25 to 64 with a Bachelor's Degree or Higher with earnings </t>
+          <t xml:space="preserve">Computer Science </t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>74150</v>
+        <v>108500</v>
       </c>
       <c r="C4" t="n">
-        <v>165.7</v>
+        <v>1597</v>
       </c>
       <c r="D4" t="n">
-        <v>60470</v>
+        <v>89310</v>
       </c>
       <c r="E4" t="n">
-        <v>171.8</v>
+        <v>2269</v>
       </c>
       <c r="F4" t="n">
-        <v>79600</v>
+        <v>120600</v>
       </c>
       <c r="G4" t="n">
-        <v>431.6</v>
+        <v>2619</v>
       </c>
       <c r="H4" t="n">
-        <v>86340</v>
+        <v>125300</v>
       </c>
       <c r="I4" t="n">
-        <v>329.9</v>
+        <v>2297</v>
       </c>
       <c r="J4" t="n">
-        <v>81580</v>
+        <v>117900</v>
       </c>
       <c r="K4" t="n">
-        <v>350.3</v>
+        <v>4350</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Science and Engineering Degrees </t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+          <t xml:space="preserve">Engineering </t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100600</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="D5" t="n">
+        <v>80370</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2238</v>
+      </c>
+      <c r="F5" t="n">
+        <v>103200</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3094</v>
+      </c>
+      <c r="H5" t="n">
+        <v>111300</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5887</v>
+      </c>
+      <c r="J5" t="n">
+        <v>106600</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2499</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Computer Science </t>
+          <t xml:space="preserve">Civil Engineering </t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>108500</v>
+        <v>99660</v>
       </c>
       <c r="C6" t="n">
-        <v>1597</v>
+        <v>1702</v>
       </c>
       <c r="D6" t="n">
-        <v>89310</v>
+        <v>80100</v>
       </c>
       <c r="E6" t="n">
-        <v>2269</v>
+        <v>1665</v>
       </c>
       <c r="F6" t="n">
-        <v>120600</v>
+        <v>105400</v>
       </c>
       <c r="G6" t="n">
-        <v>2619</v>
+        <v>2092</v>
       </c>
       <c r="H6" t="n">
-        <v>125300</v>
+        <v>123800</v>
       </c>
       <c r="I6" t="n">
-        <v>2297</v>
+        <v>3002</v>
       </c>
       <c r="J6" t="n">
-        <v>117900</v>
+        <v>111900</v>
       </c>
       <c r="K6" t="n">
-        <v>4350</v>
+        <v>6274</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Engineering </t>
+          <t xml:space="preserve">Electrical Engineering </t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>100600</v>
+        <v>121600</v>
       </c>
       <c r="C7" t="n">
-        <v>1031</v>
+        <v>1239</v>
       </c>
       <c r="D7" t="n">
-        <v>80370</v>
+        <v>95750</v>
       </c>
       <c r="E7" t="n">
-        <v>2238</v>
+        <v>2129</v>
       </c>
       <c r="F7" t="n">
-        <v>103200</v>
+        <v>124800</v>
       </c>
       <c r="G7" t="n">
-        <v>3094</v>
+        <v>2047</v>
       </c>
       <c r="H7" t="n">
-        <v>111300</v>
+        <v>139600</v>
       </c>
       <c r="I7" t="n">
-        <v>5887</v>
+        <v>3710</v>
       </c>
       <c r="J7" t="n">
-        <v>106600</v>
+        <v>131900</v>
       </c>
       <c r="K7" t="n">
-        <v>2499</v>
+        <v>3694</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Civil Engineering </t>
+          <t xml:space="preserve">Mechanical Engineering </t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>99660</v>
+        <v>106200</v>
       </c>
       <c r="C8" t="n">
-        <v>1702</v>
+        <v>957.2</v>
       </c>
       <c r="D8" t="n">
-        <v>80100</v>
+        <v>85500</v>
       </c>
       <c r="E8" t="n">
-        <v>1665</v>
+        <v>1317</v>
       </c>
       <c r="F8" t="n">
-        <v>105400</v>
+        <v>119900</v>
       </c>
       <c r="G8" t="n">
-        <v>2092</v>
+        <v>2734</v>
       </c>
       <c r="H8" t="n">
-        <v>123800</v>
+        <v>135000</v>
       </c>
       <c r="I8" t="n">
-        <v>3002</v>
+        <v>2391</v>
       </c>
       <c r="J8" t="n">
-        <v>111900</v>
+        <v>126400</v>
       </c>
       <c r="K8" t="n">
-        <v>6274</v>
+        <v>3108</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrical Engineering </t>
+          <t>Mathematics</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>121600</v>
+        <v>86560</v>
       </c>
       <c r="C9" t="n">
-        <v>1239</v>
+        <v>1476</v>
       </c>
       <c r="D9" t="n">
-        <v>95750</v>
+        <v>65170</v>
       </c>
       <c r="E9" t="n">
-        <v>2129</v>
+        <v>2484</v>
       </c>
       <c r="F9" t="n">
-        <v>124800</v>
+        <v>91600</v>
       </c>
       <c r="G9" t="n">
-        <v>2047</v>
+        <v>3870</v>
       </c>
       <c r="H9" t="n">
-        <v>139600</v>
+        <v>101800</v>
       </c>
       <c r="I9" t="n">
-        <v>3710</v>
+        <v>2176</v>
       </c>
       <c r="J9" t="n">
-        <v>131900</v>
+        <v>99990</v>
       </c>
       <c r="K9" t="n">
-        <v>3694</v>
+        <v>4439</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mechanical Engineering </t>
+          <t xml:space="preserve">Biology </t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>106200</v>
+        <v>81550</v>
       </c>
       <c r="C10" t="n">
-        <v>957.2</v>
+        <v>706.8</v>
       </c>
       <c r="D10" t="n">
-        <v>85500</v>
+        <v>60760</v>
       </c>
       <c r="E10" t="n">
-        <v>1317</v>
+        <v>786.6</v>
       </c>
       <c r="F10" t="n">
-        <v>119900</v>
+        <v>93990</v>
       </c>
       <c r="G10" t="n">
-        <v>2734</v>
+        <v>2105</v>
       </c>
       <c r="H10" t="n">
-        <v>135000</v>
+        <v>106700</v>
       </c>
       <c r="I10" t="n">
-        <v>2391</v>
+        <v>1755</v>
       </c>
       <c r="J10" t="n">
-        <v>126400</v>
+        <v>104000</v>
       </c>
       <c r="K10" t="n">
-        <v>3108</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t xml:space="preserve">Chemistry </t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>86560</v>
+        <v>94680</v>
       </c>
       <c r="C11" t="n">
-        <v>1476</v>
+        <v>2114</v>
       </c>
       <c r="D11" t="n">
-        <v>65170</v>
+        <v>61890</v>
       </c>
       <c r="E11" t="n">
-        <v>2484</v>
+        <v>1887</v>
       </c>
       <c r="F11" t="n">
-        <v>91600</v>
+        <v>100500</v>
       </c>
       <c r="G11" t="n">
-        <v>3870</v>
+        <v>2437</v>
       </c>
       <c r="H11" t="n">
-        <v>101800</v>
+        <v>121900</v>
       </c>
       <c r="I11" t="n">
-        <v>2176</v>
+        <v>4190</v>
       </c>
       <c r="J11" t="n">
-        <v>99990</v>
+        <v>110400</v>
       </c>
       <c r="K11" t="n">
-        <v>4439</v>
+        <v>6631</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biology </t>
+          <t xml:space="preserve">Psychology </t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>81550</v>
+        <v>62270</v>
       </c>
       <c r="C12" t="n">
-        <v>706.8</v>
+        <v>488.2</v>
       </c>
       <c r="D12" t="n">
-        <v>60760</v>
+        <v>50560</v>
       </c>
       <c r="E12" t="n">
-        <v>786.6</v>
+        <v>559.2</v>
       </c>
       <c r="F12" t="n">
-        <v>93990</v>
+        <v>69240</v>
       </c>
       <c r="G12" t="n">
-        <v>2105</v>
+        <v>1031</v>
       </c>
       <c r="H12" t="n">
-        <v>106700</v>
+        <v>74140</v>
       </c>
       <c r="I12" t="n">
-        <v>1755</v>
+        <v>1818</v>
       </c>
       <c r="J12" t="n">
-        <v>104000</v>
+        <v>72660</v>
       </c>
       <c r="K12" t="n">
-        <v>2100</v>
+        <v>2371</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chemistry </t>
+          <t xml:space="preserve">Economics </t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>94680</v>
+        <v>101400</v>
       </c>
       <c r="C13" t="n">
-        <v>2114</v>
+        <v>916.1</v>
       </c>
       <c r="D13" t="n">
-        <v>61890</v>
+        <v>81450</v>
       </c>
       <c r="E13" t="n">
-        <v>1887</v>
+        <v>1916</v>
       </c>
       <c r="F13" t="n">
-        <v>100500</v>
+        <v>109200</v>
       </c>
       <c r="G13" t="n">
-        <v>2437</v>
+        <v>4257</v>
       </c>
       <c r="H13" t="n">
-        <v>121900</v>
+        <v>121800</v>
       </c>
       <c r="I13" t="n">
-        <v>4190</v>
+        <v>4418</v>
       </c>
       <c r="J13" t="n">
-        <v>110400</v>
+        <v>105500</v>
       </c>
       <c r="K13" t="n">
-        <v>6631</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Psychology </t>
+          <t xml:space="preserve">Political Science </t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>62270</v>
+        <v>86380</v>
       </c>
       <c r="C14" t="n">
-        <v>488.2</v>
+        <v>1325</v>
       </c>
       <c r="D14" t="n">
-        <v>50560</v>
+        <v>67950</v>
       </c>
       <c r="E14" t="n">
-        <v>559.2</v>
+        <v>1847</v>
       </c>
       <c r="F14" t="n">
-        <v>69240</v>
+        <v>93290</v>
       </c>
       <c r="G14" t="n">
-        <v>1031</v>
+        <v>2365</v>
       </c>
       <c r="H14" t="n">
-        <v>74140</v>
+        <v>106900</v>
       </c>
       <c r="I14" t="n">
-        <v>1818</v>
+        <v>2068</v>
       </c>
       <c r="J14" t="n">
-        <v>72660</v>
+        <v>96390</v>
       </c>
       <c r="K14" t="n">
-        <v>2371</v>
+        <v>3790</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Economics </t>
+          <t xml:space="preserve">Sociology </t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>101400</v>
+        <v>63660</v>
       </c>
       <c r="C15" t="n">
-        <v>916.1</v>
+        <v>836.9</v>
       </c>
       <c r="D15" t="n">
-        <v>81450</v>
+        <v>54430</v>
       </c>
       <c r="E15" t="n">
-        <v>1916</v>
+        <v>1422</v>
       </c>
       <c r="F15" t="n">
-        <v>109200</v>
+        <v>68230</v>
       </c>
       <c r="G15" t="n">
-        <v>4257</v>
+        <v>2213</v>
       </c>
       <c r="H15" t="n">
-        <v>121800</v>
+        <v>73340</v>
       </c>
       <c r="I15" t="n">
-        <v>4418</v>
+        <v>2740</v>
       </c>
       <c r="J15" t="n">
-        <v>105500</v>
+        <v>61960</v>
       </c>
       <c r="K15" t="n">
-        <v>2352</v>
+        <v>3014</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Political Science </t>
+          <t xml:space="preserve">Nursing </t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>86380</v>
+        <v>79600</v>
       </c>
       <c r="C16" t="n">
-        <v>1325</v>
+        <v>812.7</v>
       </c>
       <c r="D16" t="n">
-        <v>67950</v>
+        <v>68220</v>
       </c>
       <c r="E16" t="n">
-        <v>1847</v>
+        <v>869.8</v>
       </c>
       <c r="F16" t="n">
-        <v>93290</v>
+        <v>81510</v>
       </c>
       <c r="G16" t="n">
-        <v>2365</v>
+        <v>869.7</v>
       </c>
       <c r="H16" t="n">
-        <v>106900</v>
+        <v>89050</v>
       </c>
       <c r="I16" t="n">
-        <v>2068</v>
+        <v>1392</v>
       </c>
       <c r="J16" t="n">
-        <v>96390</v>
+        <v>86060</v>
       </c>
       <c r="K16" t="n">
-        <v>3790</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sociology </t>
+          <t>Other Science and Engineering Degrees1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>63660</v>
+        <v>77910</v>
       </c>
       <c r="C17" t="n">
-        <v>836.9</v>
+        <v>460.3</v>
       </c>
       <c r="D17" t="n">
-        <v>54430</v>
+        <v>62030</v>
       </c>
       <c r="E17" t="n">
-        <v>1422</v>
+        <v>419.2</v>
       </c>
       <c r="F17" t="n">
-        <v>68230</v>
+        <v>85300</v>
       </c>
       <c r="G17" t="n">
-        <v>2213</v>
+        <v>727.1</v>
       </c>
       <c r="H17" t="n">
-        <v>73340</v>
+        <v>94340</v>
       </c>
       <c r="I17" t="n">
-        <v>2740</v>
+        <v>925.7</v>
       </c>
       <c r="J17" t="n">
-        <v>61960</v>
+        <v>91040</v>
       </c>
       <c r="K17" t="n">
-        <v>3014</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nursing </t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>79600</v>
-      </c>
-      <c r="C18" t="n">
-        <v>812.7</v>
-      </c>
-      <c r="D18" t="n">
-        <v>68220</v>
-      </c>
-      <c r="E18" t="n">
-        <v>869.8</v>
-      </c>
-      <c r="F18" t="n">
-        <v>81510</v>
-      </c>
-      <c r="G18" t="n">
-        <v>869.7</v>
-      </c>
-      <c r="H18" t="n">
-        <v>89050</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1392</v>
-      </c>
-      <c r="J18" t="n">
-        <v>86060</v>
-      </c>
-      <c r="K18" t="n">
-        <v>1143</v>
-      </c>
+          <t xml:space="preserve">Business Degrees </t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Other Science and Engineering Degrees1</t>
+          <t xml:space="preserve">General Business </t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>77910</v>
+        <v>80120</v>
       </c>
       <c r="C19" t="n">
-        <v>460.3</v>
+        <v>710.7</v>
       </c>
       <c r="D19" t="n">
-        <v>62030</v>
+        <v>62970</v>
       </c>
       <c r="E19" t="n">
-        <v>419.2</v>
+        <v>976.4</v>
       </c>
       <c r="F19" t="n">
-        <v>85300</v>
+        <v>84020</v>
       </c>
       <c r="G19" t="n">
-        <v>727.1</v>
+        <v>1833</v>
       </c>
       <c r="H19" t="n">
-        <v>94340</v>
+        <v>90870</v>
       </c>
       <c r="I19" t="n">
-        <v>925.7</v>
+        <v>2067</v>
       </c>
       <c r="J19" t="n">
-        <v>91040</v>
+        <v>83630</v>
       </c>
       <c r="K19" t="n">
-        <v>1095</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business Degrees </t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+          <t xml:space="preserve">Accounting </t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>84880</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1051</v>
+      </c>
+      <c r="D20" t="n">
+        <v>74020</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1131</v>
+      </c>
+      <c r="F20" t="n">
+        <v>88340</v>
+      </c>
+      <c r="G20" t="n">
+        <v>3055</v>
+      </c>
+      <c r="H20" t="n">
+        <v>93570</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1906</v>
+      </c>
+      <c r="J20" t="n">
+        <v>91440</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1830</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">General Business </t>
+          <t xml:space="preserve">Business Management and Adminstration </t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>80120</v>
+        <v>75600</v>
       </c>
       <c r="C21" t="n">
-        <v>710.7</v>
+        <v>581.2</v>
       </c>
       <c r="D21" t="n">
-        <v>62970</v>
+        <v>61790</v>
       </c>
       <c r="E21" t="n">
-        <v>976.4</v>
+        <v>871.9</v>
       </c>
       <c r="F21" t="n">
-        <v>84020</v>
+        <v>78480</v>
       </c>
       <c r="G21" t="n">
-        <v>1833</v>
+        <v>1383</v>
       </c>
       <c r="H21" t="n">
-        <v>90870</v>
+        <v>83520</v>
       </c>
       <c r="I21" t="n">
-        <v>2067</v>
+        <v>1456</v>
       </c>
       <c r="J21" t="n">
-        <v>83630</v>
+        <v>81510</v>
       </c>
       <c r="K21" t="n">
-        <v>1626</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accounting </t>
+          <t xml:space="preserve">Marketing </t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>84880</v>
+        <v>75930</v>
       </c>
       <c r="C22" t="n">
-        <v>1051</v>
+        <v>798.6</v>
       </c>
       <c r="D22" t="n">
-        <v>74020</v>
+        <v>64030</v>
       </c>
       <c r="E22" t="n">
-        <v>1131</v>
+        <v>868.8</v>
       </c>
       <c r="F22" t="n">
-        <v>88340</v>
+        <v>82870</v>
       </c>
       <c r="G22" t="n">
-        <v>3055</v>
+        <v>1970</v>
       </c>
       <c r="H22" t="n">
-        <v>93570</v>
+        <v>87340</v>
       </c>
       <c r="I22" t="n">
-        <v>1906</v>
+        <v>2789</v>
       </c>
       <c r="J22" t="n">
-        <v>91440</v>
+        <v>80380</v>
       </c>
       <c r="K22" t="n">
-        <v>1830</v>
+        <v>2732</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business Management and Adminstration </t>
+          <t xml:space="preserve">Finance </t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>75600</v>
+        <v>99900</v>
       </c>
       <c r="C23" t="n">
-        <v>581.2</v>
+        <v>1779</v>
       </c>
       <c r="D23" t="n">
-        <v>61790</v>
+        <v>81680</v>
       </c>
       <c r="E23" t="n">
-        <v>871.9</v>
+        <v>1577</v>
       </c>
       <c r="F23" t="n">
-        <v>78480</v>
+        <v>105500</v>
       </c>
       <c r="G23" t="n">
-        <v>1383</v>
+        <v>1927</v>
       </c>
       <c r="H23" t="n">
-        <v>83520</v>
+        <v>115000</v>
       </c>
       <c r="I23" t="n">
-        <v>1456</v>
+        <v>4706</v>
       </c>
       <c r="J23" t="n">
-        <v>81510</v>
+        <v>103900</v>
       </c>
       <c r="K23" t="n">
-        <v>1172</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marketing </t>
+          <t xml:space="preserve">Other Business Degrees </t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>75930</v>
+        <v>77160</v>
       </c>
       <c r="C24" t="n">
-        <v>798.6</v>
+        <v>882.2</v>
       </c>
       <c r="D24" t="n">
-        <v>64030</v>
+        <v>64070</v>
       </c>
       <c r="E24" t="n">
-        <v>868.8</v>
+        <v>1105</v>
       </c>
       <c r="F24" t="n">
-        <v>82870</v>
+        <v>82890</v>
       </c>
       <c r="G24" t="n">
-        <v>1970</v>
+        <v>1767</v>
       </c>
       <c r="H24" t="n">
-        <v>87340</v>
+        <v>88240</v>
       </c>
       <c r="I24" t="n">
-        <v>2789</v>
+        <v>2996</v>
       </c>
       <c r="J24" t="n">
-        <v>80380</v>
+        <v>82470</v>
       </c>
       <c r="K24" t="n">
-        <v>2732</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finance </t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>99900</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1779</v>
-      </c>
-      <c r="D25" t="n">
-        <v>81680</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1577</v>
-      </c>
-      <c r="F25" t="n">
-        <v>105500</v>
-      </c>
-      <c r="G25" t="n">
-        <v>1927</v>
-      </c>
-      <c r="H25" t="n">
-        <v>115000</v>
-      </c>
-      <c r="I25" t="n">
-        <v>4706</v>
-      </c>
-      <c r="J25" t="n">
-        <v>103900</v>
-      </c>
-      <c r="K25" t="n">
-        <v>2088</v>
-      </c>
+          <t xml:space="preserve">Education Degrees </t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Business Degrees </t>
+          <t>General Education</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>77160</v>
+        <v>58000</v>
       </c>
       <c r="C26" t="n">
-        <v>882.2</v>
+        <v>730.8</v>
       </c>
       <c r="D26" t="n">
-        <v>64070</v>
+        <v>50040</v>
       </c>
       <c r="E26" t="n">
-        <v>1105</v>
+        <v>734.6</v>
       </c>
       <c r="F26" t="n">
-        <v>82890</v>
+        <v>60620</v>
       </c>
       <c r="G26" t="n">
-        <v>1767</v>
+        <v>765.3</v>
       </c>
       <c r="H26" t="n">
-        <v>88240</v>
+        <v>64080</v>
       </c>
       <c r="I26" t="n">
-        <v>2996</v>
+        <v>1203</v>
       </c>
       <c r="J26" t="n">
-        <v>82470</v>
+        <v>59260</v>
       </c>
       <c r="K26" t="n">
-        <v>2493</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Education Degrees </t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+          <t>Elementary Education</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>54900</v>
+      </c>
+      <c r="C27" t="n">
+        <v>549.8</v>
+      </c>
+      <c r="D27" t="n">
+        <v>47310</v>
+      </c>
+      <c r="E27" t="n">
+        <v>671.8</v>
+      </c>
+      <c r="F27" t="n">
+        <v>56970</v>
+      </c>
+      <c r="G27" t="n">
+        <v>866.8</v>
+      </c>
+      <c r="H27" t="n">
+        <v>62980</v>
+      </c>
+      <c r="I27" t="n">
+        <v>937.9</v>
+      </c>
+      <c r="J27" t="n">
+        <v>54530</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1215</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>General Education</t>
+          <t>Other Education Degrees</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>58000</v>
+        <v>58120</v>
       </c>
       <c r="C28" t="n">
-        <v>730.8</v>
+        <v>477.6</v>
       </c>
       <c r="D28" t="n">
-        <v>50040</v>
+        <v>49860</v>
       </c>
       <c r="E28" t="n">
-        <v>734.6</v>
+        <v>571</v>
       </c>
       <c r="F28" t="n">
-        <v>60620</v>
+        <v>60390</v>
       </c>
       <c r="G28" t="n">
-        <v>765.3</v>
+        <v>739.8</v>
       </c>
       <c r="H28" t="n">
-        <v>64080</v>
+        <v>69720</v>
       </c>
       <c r="I28" t="n">
-        <v>1203</v>
+        <v>1140</v>
       </c>
       <c r="J28" t="n">
-        <v>59260</v>
+        <v>58370</v>
       </c>
       <c r="K28" t="n">
-        <v>1631</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Elementary Education</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>54900</v>
-      </c>
-      <c r="C29" t="n">
-        <v>549.8</v>
-      </c>
-      <c r="D29" t="n">
-        <v>47310</v>
-      </c>
-      <c r="E29" t="n">
-        <v>671.8</v>
-      </c>
-      <c r="F29" t="n">
-        <v>56970</v>
-      </c>
-      <c r="G29" t="n">
-        <v>866.8</v>
-      </c>
-      <c r="H29" t="n">
-        <v>62980</v>
-      </c>
-      <c r="I29" t="n">
-        <v>937.9</v>
-      </c>
-      <c r="J29" t="n">
-        <v>54530</v>
-      </c>
-      <c r="K29" t="n">
-        <v>1215</v>
-      </c>
+          <t xml:space="preserve">Arts, Humanities and Other Degrees </t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Other Education Degrees</t>
+          <t xml:space="preserve">Communications </t>
         </is>
       </c>
       <c r="B30" t="n">
+        <v>67840</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1017</v>
+      </c>
+      <c r="D30" t="n">
         <v>58120</v>
       </c>
-      <c r="C30" t="n">
-        <v>477.6</v>
-      </c>
-      <c r="D30" t="n">
-        <v>49860</v>
-      </c>
       <c r="E30" t="n">
-        <v>571</v>
+        <v>1500</v>
       </c>
       <c r="F30" t="n">
-        <v>60390</v>
+        <v>74780</v>
       </c>
       <c r="G30" t="n">
-        <v>739.8</v>
+        <v>1411</v>
       </c>
       <c r="H30" t="n">
-        <v>69720</v>
+        <v>80000</v>
       </c>
       <c r="I30" t="n">
-        <v>1140</v>
+        <v>2566</v>
       </c>
       <c r="J30" t="n">
-        <v>58370</v>
+        <v>71880</v>
       </c>
       <c r="K30" t="n">
-        <v>1298</v>
+        <v>2071</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arts, Humanities and Other Degrees </t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+          <t xml:space="preserve">English Language and Literature </t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>65060</v>
+      </c>
+      <c r="C31" t="n">
+        <v>927</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51010</v>
+      </c>
+      <c r="E31" t="n">
+        <v>914.2</v>
+      </c>
+      <c r="F31" t="n">
+        <v>69620</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1552</v>
+      </c>
+      <c r="H31" t="n">
+        <v>76620</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1485</v>
+      </c>
+      <c r="J31" t="n">
+        <v>71770</v>
+      </c>
+      <c r="K31" t="n">
+        <v>2599</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Communications </t>
+          <t xml:space="preserve">Liberal Arts </t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>67840</v>
+        <v>61380</v>
       </c>
       <c r="C32" t="n">
-        <v>1017</v>
+        <v>1044</v>
       </c>
       <c r="D32" t="n">
-        <v>58120</v>
+        <v>47960</v>
       </c>
       <c r="E32" t="n">
-        <v>1500</v>
+        <v>1912</v>
       </c>
       <c r="F32" t="n">
-        <v>74780</v>
+        <v>64260</v>
       </c>
       <c r="G32" t="n">
-        <v>1411</v>
+        <v>2253</v>
       </c>
       <c r="H32" t="n">
-        <v>80000</v>
+        <v>73070</v>
       </c>
       <c r="I32" t="n">
-        <v>2566</v>
+        <v>3740</v>
       </c>
       <c r="J32" t="n">
-        <v>71880</v>
+        <v>64270</v>
       </c>
       <c r="K32" t="n">
-        <v>2071</v>
+        <v>3313</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">English Language and Literature </t>
+          <t xml:space="preserve">History </t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>65060</v>
+        <v>73560</v>
       </c>
       <c r="C33" t="n">
-        <v>927</v>
+        <v>1006</v>
       </c>
       <c r="D33" t="n">
-        <v>51010</v>
+        <v>54240</v>
       </c>
       <c r="E33" t="n">
-        <v>914.2</v>
+        <v>1021</v>
       </c>
       <c r="F33" t="n">
-        <v>69620</v>
+        <v>76160</v>
       </c>
       <c r="G33" t="n">
-        <v>1552</v>
+        <v>1665</v>
       </c>
       <c r="H33" t="n">
-        <v>76620</v>
+        <v>90570</v>
       </c>
       <c r="I33" t="n">
-        <v>1485</v>
+        <v>2950</v>
       </c>
       <c r="J33" t="n">
-        <v>71770</v>
+        <v>86240</v>
       </c>
       <c r="K33" t="n">
-        <v>2599</v>
+        <v>3154</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liberal Arts </t>
+          <t xml:space="preserve">Fine Arts </t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>61380</v>
+        <v>53450</v>
       </c>
       <c r="C34" t="n">
-        <v>1044</v>
+        <v>1303</v>
       </c>
       <c r="D34" t="n">
-        <v>47960</v>
+        <v>42220</v>
       </c>
       <c r="E34" t="n">
-        <v>1912</v>
+        <v>1850</v>
       </c>
       <c r="F34" t="n">
-        <v>64260</v>
+        <v>57920</v>
       </c>
       <c r="G34" t="n">
-        <v>2253</v>
+        <v>2891</v>
       </c>
       <c r="H34" t="n">
-        <v>73070</v>
+        <v>62410</v>
       </c>
       <c r="I34" t="n">
-        <v>3740</v>
+        <v>1870</v>
       </c>
       <c r="J34" t="n">
-        <v>64270</v>
+        <v>53300</v>
       </c>
       <c r="K34" t="n">
-        <v>3313</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">History </t>
+          <t xml:space="preserve">Commerical Art and Graphic Design </t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>73560</v>
+        <v>59770</v>
       </c>
       <c r="C35" t="n">
-        <v>1006</v>
+        <v>1049</v>
       </c>
       <c r="D35" t="n">
-        <v>54240</v>
+        <v>52290</v>
       </c>
       <c r="E35" t="n">
-        <v>1021</v>
+        <v>1175</v>
       </c>
       <c r="F35" t="n">
-        <v>76160</v>
+        <v>66830</v>
       </c>
       <c r="G35" t="n">
-        <v>1665</v>
+        <v>2508</v>
       </c>
       <c r="H35" t="n">
-        <v>90570</v>
+        <v>68560</v>
       </c>
       <c r="I35" t="n">
-        <v>2950</v>
+        <v>4018</v>
       </c>
       <c r="J35" t="n">
-        <v>86240</v>
+        <v>54740</v>
       </c>
       <c r="K35" t="n">
-        <v>3154</v>
+        <v>4040</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fine Arts </t>
+          <t xml:space="preserve">Family and Consumer Sciences </t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>53450</v>
+        <v>52850</v>
       </c>
       <c r="C36" t="n">
-        <v>1303</v>
+        <v>951.6</v>
       </c>
       <c r="D36" t="n">
-        <v>42220</v>
+        <v>47190</v>
       </c>
       <c r="E36" t="n">
-        <v>1850</v>
+        <v>1567</v>
       </c>
       <c r="F36" t="n">
-        <v>57920</v>
+        <v>57560</v>
       </c>
       <c r="G36" t="n">
-        <v>2891</v>
+        <v>4088</v>
       </c>
       <c r="H36" t="n">
-        <v>62410</v>
+        <v>60360</v>
       </c>
       <c r="I36" t="n">
-        <v>1870</v>
+        <v>3569</v>
       </c>
       <c r="J36" t="n">
-        <v>53300</v>
+        <v>52130</v>
       </c>
       <c r="K36" t="n">
-        <v>2358</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commerical Art and Graphic Design </t>
+          <t>Physical Fitness, Parks, Recreation, and Leisure</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>59770</v>
+        <v>61580</v>
       </c>
       <c r="C37" t="n">
-        <v>1049</v>
+        <v>691.3</v>
       </c>
       <c r="D37" t="n">
-        <v>52290</v>
+        <v>52250</v>
       </c>
       <c r="E37" t="n">
-        <v>1175</v>
+        <v>986.2</v>
       </c>
       <c r="F37" t="n">
-        <v>66830</v>
+        <v>70740</v>
       </c>
       <c r="G37" t="n">
-        <v>2508</v>
+        <v>2268</v>
       </c>
       <c r="H37" t="n">
-        <v>68560</v>
+        <v>76910</v>
       </c>
       <c r="I37" t="n">
-        <v>4018</v>
+        <v>2600</v>
       </c>
       <c r="J37" t="n">
-        <v>54740</v>
+        <v>64550</v>
       </c>
       <c r="K37" t="n">
-        <v>4040</v>
+        <v>2992</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Family and Consumer Sciences </t>
+          <t>Criminal Justice and Fire Protection</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>52850</v>
+        <v>64690</v>
       </c>
       <c r="C38" t="n">
-        <v>951.6</v>
+        <v>809.2</v>
       </c>
       <c r="D38" t="n">
-        <v>47190</v>
+        <v>52450</v>
       </c>
       <c r="E38" t="n">
-        <v>1567</v>
+        <v>758.3</v>
       </c>
       <c r="F38" t="n">
-        <v>57560</v>
+        <v>72130</v>
       </c>
       <c r="G38" t="n">
-        <v>4088</v>
+        <v>1370</v>
       </c>
       <c r="H38" t="n">
-        <v>60360</v>
+        <v>79040</v>
       </c>
       <c r="I38" t="n">
-        <v>3569</v>
+        <v>3245</v>
       </c>
       <c r="J38" t="n">
-        <v>52130</v>
+        <v>68800</v>
       </c>
       <c r="K38" t="n">
-        <v>2545</v>
+        <v>3884</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Physical Fitness, Parks, Recreation, and Leisure</t>
+          <t xml:space="preserve">Social Work </t>
         </is>
       </c>
       <c r="B39" t="n">
+        <v>55060</v>
+      </c>
+      <c r="C39" t="n">
+        <v>838</v>
+      </c>
+      <c r="D39" t="n">
+        <v>48040</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1623</v>
+      </c>
+      <c r="F39" t="n">
+        <v>59880</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1726</v>
+      </c>
+      <c r="H39" t="n">
         <v>61580</v>
       </c>
-      <c r="C39" t="n">
-        <v>691.3</v>
-      </c>
-      <c r="D39" t="n">
-        <v>52250</v>
-      </c>
-      <c r="E39" t="n">
-        <v>986.2</v>
-      </c>
-      <c r="F39" t="n">
-        <v>70740</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2268</v>
-      </c>
-      <c r="H39" t="n">
-        <v>76910</v>
-      </c>
       <c r="I39" t="n">
-        <v>2600</v>
+        <v>1888</v>
       </c>
       <c r="J39" t="n">
-        <v>64550</v>
+        <v>56970</v>
       </c>
       <c r="K39" t="n">
-        <v>2992</v>
+        <v>3012</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Criminal Justice and Fire Protection</t>
+          <t xml:space="preserve">Other Degrees </t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>64690</v>
+        <v>62100</v>
       </c>
       <c r="C40" t="n">
-        <v>809.2</v>
+        <v>419.6</v>
       </c>
       <c r="D40" t="n">
-        <v>52450</v>
+        <v>50880</v>
       </c>
       <c r="E40" t="n">
-        <v>758.3</v>
+        <v>501.4</v>
       </c>
       <c r="F40" t="n">
-        <v>72130</v>
+        <v>68090</v>
       </c>
       <c r="G40" t="n">
-        <v>1370</v>
+        <v>970.4</v>
       </c>
       <c r="H40" t="n">
-        <v>79040</v>
+        <v>74100</v>
       </c>
       <c r="I40" t="n">
-        <v>3245</v>
+        <v>1281</v>
       </c>
       <c r="J40" t="n">
-        <v>68800</v>
+        <v>64780</v>
       </c>
       <c r="K40" t="n">
-        <v>3884</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Work </t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>55060</v>
-      </c>
-      <c r="C41" t="n">
-        <v>838</v>
-      </c>
-      <c r="D41" t="n">
-        <v>48040</v>
-      </c>
-      <c r="E41" t="n">
-        <v>1623</v>
-      </c>
-      <c r="F41" t="n">
-        <v>59880</v>
-      </c>
-      <c r="G41" t="n">
-        <v>1726</v>
-      </c>
-      <c r="H41" t="n">
-        <v>61580</v>
-      </c>
-      <c r="I41" t="n">
-        <v>1888</v>
-      </c>
-      <c r="J41" t="n">
-        <v>56970</v>
-      </c>
-      <c r="K41" t="n">
-        <v>3012</v>
-      </c>
+          <t>Source: U.S. Census Bureau, 2022 American Community Survey, 1-year estimates. For more information, refer to &lt;www.census.gov/acs&gt;.</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Degrees </t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>62100</v>
-      </c>
-      <c r="C42" t="n">
-        <v>419.6</v>
-      </c>
-      <c r="D42" t="n">
-        <v>50880</v>
-      </c>
-      <c r="E42" t="n">
-        <v>501.4</v>
-      </c>
-      <c r="F42" t="n">
-        <v>68090</v>
-      </c>
-      <c r="G42" t="n">
-        <v>970.4</v>
-      </c>
-      <c r="H42" t="n">
-        <v>74100</v>
-      </c>
-      <c r="I42" t="n">
-        <v>1281</v>
-      </c>
-      <c r="J42" t="n">
-        <v>64780</v>
-      </c>
-      <c r="K42" t="n">
-        <v>1217</v>
-      </c>
+          <t>The Census Bureau has reviewed this data product to ensure appropriate access, use, and disclosure avoidance protection of the confidential source data used to produce this product (Data Management System (DMS) number: P-001-0000001262, Disclosure Review Board (DRB) approval number: CBDRB-FY23-SEHSD003-068.</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Source: U.S. Census Bureau, 2022 American Community Survey, 1-year estimates. For more information, refer to &lt;www.census.gov/acs&gt;.</t>
+          <t>Note: 1. Science and Engineering related fields are included within the "other science and engineering degrees" category.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -1955,40 +1899,6 @@
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>The Census Bureau has reviewed this data product to ensure appropriate access, use, and disclosure avoidance protection of the confidential source data used to produce this product (Data Management System (DMS) number: P-001-0000001262, Disclosure Review Board (DRB) approval number: CBDRB-FY23-SEHSD003-068.</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Note: 1. Science and Engineering related fields are included within the "other science and engineering degrees" category.</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>